<commit_message>
docs(qa): fix testing progress documentation
</commit_message>
<xml_diff>
--- a/docs/qa-testing/Testing Progress(7_12_2026).xlsx
+++ b/docs/qa-testing/Testing Progress(7_12_2026).xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabreal\Downloads\ahahjhaa\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Users\Gabreal\Games\MyPersonalHell(GitHub)\schooools\Accounting-AI-Financial-Assistant\docs\qa-testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F76A97F-6006-45A9-9EC5-4F9B7F0912CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F257CDE-1ADA-4030-85E0-0D5288655670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="18870" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Testing" sheetId="2" r:id="rId1"/>
@@ -91,9 +91,6 @@
     <t>Download generated files</t>
   </si>
   <si>
-    <t>Generated files download and open successfully.</t>
-  </si>
-  <si>
     <t>Simple settings/preferences</t>
   </si>
   <si>
@@ -110,6 +107,9 @@
   </si>
   <si>
     <t>Feature 7/12/2026</t>
+  </si>
+  <si>
+    <t>Generated files not yet implemented</t>
   </si>
 </sst>
 </file>
@@ -638,7 +638,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>0</v>
@@ -661,7 +661,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -675,7 +675,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -689,7 +689,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -703,7 +703,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -745,7 +745,7 @@
         <v>18</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -767,24 +767,24 @@
         <v>21</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D10" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="C11" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="D11" s="9" t="b">
         <v>0</v>

</xml_diff>